<commit_message>
Update remarks: 911 partial payment, 216 awaiting booking form
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UCaoJyXjiybYwzoEQ19eV5
</commit_message>
<xml_diff>
--- a/outputs/Pending_Receivables_Remarks_14-Oct-2026.xlsx
+++ b/outputs/Pending_Receivables_Remarks_14-Oct-2026.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>More than 24% paid so far. The client is still within the payment period.</t>
+          <t>More than 24% paid so far. Awaiting the booking form. The client is still within the payment period.</t>
         </is>
       </c>
     </row>
@@ -638,12 +638,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Partially paid</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Payment completed. The POP has already been shared with you.</t>
+          <t>AED 175K was paid yesterday (13-Oct-2026). The remaining AED 175K will be sent today (14-Oct-2026).</t>
         </is>
       </c>
     </row>

</xml_diff>